<commit_message>
Updated with Dushin IEP/ELLs
</commit_message>
<xml_diff>
--- a/Global/October CMA/Global October CMA Data.xlsx
+++ b/Global/October CMA/Global October CMA Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coledushin/Documents/GWHS/Global/October CMA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C8CC1F-8467-D04E-9B6D-64E1F9F60BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDD2B7D-C4C4-A44C-9DBC-0453DA749751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="15520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2818,33 +2818,6 @@
   </cellStyles>
   <dxfs count="31">
     <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF3F4A58"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FFBB463C"/>
       </font>
@@ -2854,6 +2827,12 @@
           <bgColor rgb="FFFFD9D6"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2875,6 +2854,27 @@
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF3F4A58"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -3206,10 +3206,6 @@
 </FeaturePropertyBags>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Scores" displayName="Scores" ref="A1:AD82">
   <tableColumns count="30">
@@ -3217,9 +3213,9 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="First"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Last"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Class"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Period" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ELL" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Period" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ELL" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="4"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MC"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="CRQ"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Final"/>
@@ -3304,7 +3300,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="#"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Framework"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Specifications"/>
-    <tableColumn id="4" xr3:uid="{37E3D24F-9292-BD43-B3FC-16D6A7D0B3AB}" name="Concatenated" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{37E3D24F-9292-BD43-B3FC-16D6A7D0B3AB}" name="Concatenated" dataDxfId="1">
       <calculatedColumnFormula>_xlfn.CONCAT(Table3[[#This Row],['#]],": ",Table3[[#This Row],[Framework]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7344,7 +7340,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H40" s="3">
         <f t="shared" si="2"/>
@@ -7635,7 +7631,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H43" s="3">
         <f t="shared" si="2"/>
@@ -7829,7 +7825,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H45" s="3">
         <f t="shared" si="2"/>
@@ -8116,7 +8112,7 @@
         <v>0</v>
       </c>
       <c r="G48" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H48" s="3">
         <f t="shared" si="2"/>
@@ -8504,7 +8500,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" s="3">
         <f t="shared" si="2"/>
@@ -8698,7 +8694,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H54" s="3">
         <f t="shared" si="2"/>
@@ -8892,7 +8888,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H56" s="3">
         <f t="shared" si="2"/>
@@ -9177,7 +9173,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H59" s="3">
         <f t="shared" si="2"/>
@@ -10144,7 +10140,7 @@
         <v>4</v>
       </c>
       <c r="F69" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G69" s="10" t="b">
         <v>0</v>
@@ -10341,7 +10337,7 @@
         <v>0</v>
       </c>
       <c r="G71" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H71" s="3">
         <f t="shared" si="2"/>
@@ -11016,7 +11012,7 @@
         <v>0</v>
       </c>
       <c r="G78" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H78" s="3">
         <f t="shared" si="2"/>
@@ -11307,7 +11303,7 @@
         <v>0</v>
       </c>
       <c r="G81" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H81" s="3">
         <f t="shared" si="2"/>
@@ -11404,7 +11400,7 @@
         <v>0</v>
       </c>
       <c r="G82" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H82" s="3">
         <f t="shared" si="2"/>
@@ -11481,7 +11477,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="K2:R82">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>W2=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12171,6 +12167,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>

</xml_diff>